<commit_message>
Add temp_manager_update, Update Excel template and restrict job fetch SQL for testing.
</commit_message>
<xml_diff>
--- a/Jobs/Tasks/FileProcess/ManagerUpdateDataExcel.xlsx
+++ b/Jobs/Tasks/FileProcess/ManagerUpdateDataExcel.xlsx
@@ -19,23 +19,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>AGT002</t>
   </si>
   <si>
-    <t>2026-01-05</t>
-  </si>
-  <si>
     <t>AgentCode</t>
   </si>
   <si>
     <t>SupervisorCode</t>
   </si>
   <si>
-    <t>AG100</t>
-  </si>
-  <si>
     <t>EffectiveDateOfChange</t>
   </si>
   <si>
@@ -46,6 +40,9 @@
   </si>
   <si>
     <t>2026-01-06</t>
+  </si>
+  <si>
+    <t>UH26020300005</t>
   </si>
 </sst>
 </file>
@@ -104,11 +101,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,35 +421,35 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
-        <v>1</v>
+      <c r="C2" s="2">
+        <v>46066</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add bulk agent status update via temp_status_update table
</commit_message>
<xml_diff>
--- a/Jobs/Tasks/FileProcess/ManagerUpdateDataExcel.xlsx
+++ b/Jobs/Tasks/FileProcess/ManagerUpdateDataExcel.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>AGT002</t>
   </si>
@@ -33,16 +33,7 @@
     <t>EffectiveDateOfChange</t>
   </si>
   <si>
-    <t>AG150</t>
-  </si>
-  <si>
-    <t>AG20534</t>
-  </si>
-  <si>
-    <t>2026-01-06</t>
-  </si>
-  <si>
-    <t>UH26020300005</t>
+    <t>AG2602151625004</t>
   </si>
 </sst>
 </file>
@@ -411,10 +402,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.36328125" bestFit="1" customWidth="1"/>
   </cols>
@@ -432,24 +423,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2">
-        <v>46066</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
+        <v>46070</v>
       </c>
     </row>
   </sheetData>

</xml_diff>